<commit_message>
Add Nielsen competitive, pack-size & state readout (national Urban, May'26)
Sourced from an unmerged prior branch (claude/retail-channel-performance-hz0q8h)
that had richer Nielsen slides (competitor brand rankings, Mamaearth pack-size
mix, zone/state share) than the MT-vs-GT panel used so far. Adds it as a THIRD
independent dataset across all three deliverables:

- dashboard: new NIELSEN_COMP object + nielsenCompHtml() card on Market Share
  tab, clearly labeled as national-Urban/no-channel-split/May'26 vintage,
  never merged with D or RETAIL_AUDIT
- Excel: new "Nielsen Competitor & State" sheet + one extra action-tracker row
- PPT: two new slides (Competitive Landscape, Pack-Size & State White Space)

Key derived insight: Uttar Pradesh and Maharashtra are the largest
under-penetrated states across both Facewash and Shampoo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GvaoD8EEUD7VSbiFjT5PH1
</commit_message>
<xml_diff>
--- a/reports/MT_vs_GT_Analysis.xlsx
+++ b/reports/MT_vs_GT_Analysis.xlsx
@@ -7,8 +7,9 @@
     <sheet name="Raw Data - Facewash" sheetId="1" r:id="rId1"/>
     <sheet name="Raw Data - Shampoo" sheetId="2" r:id="rId2"/>
     <sheet name="Pack Mix - Shampoo" sheetId="3" r:id="rId3"/>
-    <sheet name="MT vs GT Summary" sheetId="4" r:id="rId4"/>
-    <sheet name="Action Tracker" sheetId="5" r:id="rId5"/>
+    <sheet name="Nielsen Competitor &amp; State" sheetId="4" r:id="rId4"/>
+    <sheet name="MT vs GT Summary" sheetId="5" r:id="rId5"/>
+    <sheet name="Action Tracker" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -2527,6 +2528,1218 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NIELSEN COMPETITIVE, PACK &amp; STATE READOUT — National Urban, May'26 (separate source, not MT/GT split)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FACEWASH — Top competitors (National Urban Nielsen MS Val, May'26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rank</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brand</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value (Cr)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YoY Val %</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS Val %</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MoM (bps)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YoY (bps)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wtd Dist %</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>1</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Himalaya</t>
+        </is>
+      </c>
+      <c r="C5" s="0">
+        <v>17.9</v>
+      </c>
+      <c r="D5" s="0">
+        <v>-2</v>
+      </c>
+      <c r="E5" s="0">
+        <v>22</v>
+      </c>
+      <c r="F5" s="0">
+        <v>20</v>
+      </c>
+      <c r="G5" s="0">
+        <v>-328</v>
+      </c>
+      <c r="H5" s="0">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>2</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Garnier</t>
+        </is>
+      </c>
+      <c r="C6" s="0">
+        <v>11.8</v>
+      </c>
+      <c r="D6" s="0">
+        <v>17</v>
+      </c>
+      <c r="E6" s="0">
+        <v>14</v>
+      </c>
+      <c r="F6" s="0">
+        <v>43</v>
+      </c>
+      <c r="G6" s="0">
+        <v>55</v>
+      </c>
+      <c r="H6" s="0">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>3</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pond's</t>
+        </is>
+      </c>
+      <c r="C7" s="0">
+        <v>11.4</v>
+      </c>
+      <c r="D7" s="0">
+        <v>8</v>
+      </c>
+      <c r="E7" s="0">
+        <v>14</v>
+      </c>
+      <c r="F7" s="0">
+        <v>-114</v>
+      </c>
+      <c r="G7" s="0">
+        <v>-61</v>
+      </c>
+      <c r="H7" s="0">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4">
+        <v>4</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mamaearth</t>
+        </is>
+      </c>
+      <c r="C8" s="4">
+        <v>9.6</v>
+      </c>
+      <c r="D8" s="4">
+        <v>54</v>
+      </c>
+      <c r="E8" s="4">
+        <v>12</v>
+      </c>
+      <c r="F8" s="4">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>311</v>
+      </c>
+      <c r="H8" s="4">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>5</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clean &amp; Clear</t>
+        </is>
+      </c>
+      <c r="C9" s="0">
+        <v>6.3</v>
+      </c>
+      <c r="D9" s="0">
+        <v>16</v>
+      </c>
+      <c r="E9" s="0">
+        <v>8</v>
+      </c>
+      <c r="F9" s="0">
+        <v>3</v>
+      </c>
+      <c r="G9" s="0">
+        <v>22</v>
+      </c>
+      <c r="H9" s="0">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>6</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Joy</t>
+        </is>
+      </c>
+      <c r="C10" s="0">
+        <v>4.9</v>
+      </c>
+      <c r="D10" s="0">
+        <v>7</v>
+      </c>
+      <c r="E10" s="0">
+        <v>6</v>
+      </c>
+      <c r="F10" s="0">
+        <v>7</v>
+      </c>
+      <c r="G10" s="0">
+        <v>-30</v>
+      </c>
+      <c r="H10" s="0">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0">
+        <v>7</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lakme</t>
+        </is>
+      </c>
+      <c r="C11" s="0">
+        <v>3.1</v>
+      </c>
+      <c r="D11" s="0">
+        <v>23</v>
+      </c>
+      <c r="E11" s="0">
+        <v>4</v>
+      </c>
+      <c r="F11" s="0">
+        <v>60</v>
+      </c>
+      <c r="G11" s="0">
+        <v>31</v>
+      </c>
+      <c r="H11" s="0">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0">
+        <v>8</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nivea Men</t>
+        </is>
+      </c>
+      <c r="C12" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="D12" s="0">
+        <v>-2</v>
+      </c>
+      <c r="E12" s="0">
+        <v>4</v>
+      </c>
+      <c r="F12" s="0">
+        <v>-7</v>
+      </c>
+      <c r="G12" s="0">
+        <v>-54</v>
+      </c>
+      <c r="H12" s="0">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0">
+        <v>9</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simple</t>
+        </is>
+      </c>
+      <c r="C13" s="0">
+        <v>1.9</v>
+      </c>
+      <c r="D13" s="0"/>
+      <c r="E13" s="0">
+        <v>2</v>
+      </c>
+      <c r="F13" s="0">
+        <v>36</v>
+      </c>
+      <c r="G13" s="0">
+        <v>223</v>
+      </c>
+      <c r="H13" s="0">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Derma Co</t>
+        </is>
+      </c>
+      <c r="C14" s="4">
+        <v>0.606</v>
+      </c>
+      <c r="D14" s="4">
+        <v>3940</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="F14" s="4">
+        <v>6</v>
+      </c>
+      <c r="G14" s="4">
+        <v>71</v>
+      </c>
+      <c r="H14" s="4">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SHAMPOO — Top competitors (National Urban Nielsen MS Val, May'26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rank</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brand</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value (Cr)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YoY Val %</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS Val %</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MoM (bps)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YoY (bps)</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wtd Dist %</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0">
+        <v>1</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dove</t>
+        </is>
+      </c>
+      <c r="C18" s="0">
+        <v>29.6</v>
+      </c>
+      <c r="D18" s="0">
+        <v>7</v>
+      </c>
+      <c r="E18" s="0">
+        <v>18</v>
+      </c>
+      <c r="F18" s="0">
+        <v>170</v>
+      </c>
+      <c r="G18" s="0">
+        <v>20</v>
+      </c>
+      <c r="H18" s="0">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0">
+        <v>2</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L'Oreal Paris</t>
+        </is>
+      </c>
+      <c r="C19" s="0">
+        <v>22.1</v>
+      </c>
+      <c r="D19" s="0">
+        <v>20</v>
+      </c>
+      <c r="E19" s="0">
+        <v>13</v>
+      </c>
+      <c r="F19" s="0">
+        <v>70</v>
+      </c>
+      <c r="G19" s="0">
+        <v>130</v>
+      </c>
+      <c r="H19" s="0">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0">
+        <v>3</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Head &amp; Shoulders</t>
+        </is>
+      </c>
+      <c r="C20" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="D20" s="0">
+        <v>-8</v>
+      </c>
+      <c r="E20" s="0">
+        <v>11</v>
+      </c>
+      <c r="F20" s="0">
+        <v>130</v>
+      </c>
+      <c r="G20" s="0">
+        <v>200</v>
+      </c>
+      <c r="H20" s="0">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0">
+        <v>4</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tresemme</t>
+        </is>
+      </c>
+      <c r="C21" s="0">
+        <v>17.3</v>
+      </c>
+      <c r="D21" s="0">
+        <v>25</v>
+      </c>
+      <c r="E21" s="0">
+        <v>10</v>
+      </c>
+      <c r="F21" s="0">
+        <v>90</v>
+      </c>
+      <c r="G21" s="0">
+        <v>140</v>
+      </c>
+      <c r="H21" s="0">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0">
+        <v>5</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clinic Plus</t>
+        </is>
+      </c>
+      <c r="C22" s="0">
+        <v>16.7</v>
+      </c>
+      <c r="D22" s="0">
+        <v>14</v>
+      </c>
+      <c r="E22" s="0">
+        <v>10</v>
+      </c>
+      <c r="F22" s="0">
+        <v>30</v>
+      </c>
+      <c r="G22" s="0">
+        <v>50</v>
+      </c>
+      <c r="H22" s="0">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0">
+        <v>6</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sunsilk</t>
+        </is>
+      </c>
+      <c r="C23" s="0">
+        <v>14.8</v>
+      </c>
+      <c r="D23" s="0">
+        <v>-7</v>
+      </c>
+      <c r="E23" s="0">
+        <v>9</v>
+      </c>
+      <c r="F23" s="0">
+        <v>0</v>
+      </c>
+      <c r="G23" s="0">
+        <v>150</v>
+      </c>
+      <c r="H23" s="0">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4">
+        <v>7</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mamaearth</t>
+        </is>
+      </c>
+      <c r="C24" s="4">
+        <v>6.5</v>
+      </c>
+      <c r="D24" s="4">
+        <v>64</v>
+      </c>
+      <c r="E24" s="4">
+        <v>4</v>
+      </c>
+      <c r="F24" s="4">
+        <v>30</v>
+      </c>
+      <c r="G24" s="4">
+        <v>130</v>
+      </c>
+      <c r="H24" s="4">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0">
+        <v>8</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pantene</t>
+        </is>
+      </c>
+      <c r="C25" s="0">
+        <v>6.5</v>
+      </c>
+      <c r="D25" s="0">
+        <v>-4</v>
+      </c>
+      <c r="E25" s="0">
+        <v>4</v>
+      </c>
+      <c r="F25" s="0">
+        <v>30</v>
+      </c>
+      <c r="G25" s="0">
+        <v>50</v>
+      </c>
+      <c r="H25" s="0">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0">
+        <v>9</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Himalaya</t>
+        </is>
+      </c>
+      <c r="C26" s="0">
+        <v>5.7</v>
+      </c>
+      <c r="D26" s="0">
+        <v>2</v>
+      </c>
+      <c r="E26" s="0">
+        <v>3</v>
+      </c>
+      <c r="F26" s="0">
+        <v>40</v>
+      </c>
+      <c r="G26" s="0">
+        <v>20</v>
+      </c>
+      <c r="H26" s="0">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mamaearth Facewash — pack size (National Urban, May'26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rank</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pack</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contribution %</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MoM (bps)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YoY (bps)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value (Cr)</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YoY Growth %</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4">
+        <v>1</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">150ml</t>
+        </is>
+      </c>
+      <c r="C30" s="4">
+        <v>58</v>
+      </c>
+      <c r="D30" s="4">
+        <v>-40</v>
+      </c>
+      <c r="E30" s="4">
+        <v>290</v>
+      </c>
+      <c r="F30" s="4">
+        <v>5.53</v>
+      </c>
+      <c r="G30" s="4">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4">
+        <v>2</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100ml</t>
+        </is>
+      </c>
+      <c r="C31" s="4">
+        <v>21</v>
+      </c>
+      <c r="D31" s="4">
+        <v>-40</v>
+      </c>
+      <c r="E31" s="4">
+        <v>-60</v>
+      </c>
+      <c r="F31" s="4">
+        <v>1.96</v>
+      </c>
+      <c r="G31" s="4">
+        <v>-11</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4">
+        <v>3</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">200ml</t>
+        </is>
+      </c>
+      <c r="C32" s="4">
+        <v>11</v>
+      </c>
+      <c r="D32" s="4">
+        <v>90</v>
+      </c>
+      <c r="E32" s="4">
+        <v>130</v>
+      </c>
+      <c r="F32" s="4">
+        <v>1.06</v>
+      </c>
+      <c r="G32" s="4"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4">
+        <v>4</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">50ml</t>
+        </is>
+      </c>
+      <c r="C33" s="4">
+        <v>11</v>
+      </c>
+      <c r="D33" s="4">
+        <v>-10</v>
+      </c>
+      <c r="E33" s="4">
+        <v>50</v>
+      </c>
+      <c r="F33" s="4">
+        <v>1.01</v>
+      </c>
+      <c r="G33" s="4">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4">
+        <v>5</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">250ml</t>
+        </is>
+      </c>
+      <c r="C34" s="4">
+        <v>0</v>
+      </c>
+      <c r="D34" s="4">
+        <v>0</v>
+      </c>
+      <c r="E34" s="4">
+        <v>-80</v>
+      </c>
+      <c r="F34" s="4">
+        <v>0.04</v>
+      </c>
+      <c r="G34" s="4">
+        <v>-94</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High-contribution, low-share states — distribution white space (May'26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Category</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">State</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contribution to Category %</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">May'26 Share %</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MoM (bps)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facewash</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="C38" s="3">
+        <v>15</v>
+      </c>
+      <c r="D38" s="3">
+        <v>6</v>
+      </c>
+      <c r="E38" s="3">
+        <v>-122</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facewash</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maharashtra</t>
+        </is>
+      </c>
+      <c r="C39" s="3">
+        <v>14</v>
+      </c>
+      <c r="D39" s="3">
+        <v>6</v>
+      </c>
+      <c r="E39" s="3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facewash</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Bengal</t>
+        </is>
+      </c>
+      <c r="C40" s="3">
+        <v>8</v>
+      </c>
+      <c r="D40" s="3">
+        <v>5</v>
+      </c>
+      <c r="E40" s="3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facewash</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delhi</t>
+        </is>
+      </c>
+      <c r="C41" s="0">
+        <v>8</v>
+      </c>
+      <c r="D41" s="0">
+        <v>9</v>
+      </c>
+      <c r="E41" s="0">
+        <v>-42</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facewash</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Haryana</t>
+        </is>
+      </c>
+      <c r="C42" s="0">
+        <v>6</v>
+      </c>
+      <c r="D42" s="0">
+        <v>8</v>
+      </c>
+      <c r="E42" s="0">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facewash</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Madhya Pradesh</t>
+        </is>
+      </c>
+      <c r="C43" s="0">
+        <v>6</v>
+      </c>
+      <c r="D43" s="0">
+        <v>7</v>
+      </c>
+      <c r="E43" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facewash</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bihar</t>
+        </is>
+      </c>
+      <c r="C44" s="0">
+        <v>6</v>
+      </c>
+      <c r="D44" s="0">
+        <v>5</v>
+      </c>
+      <c r="E44" s="0">
+        <v>-15</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facewash</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gujarat</t>
+        </is>
+      </c>
+      <c r="C45" s="0">
+        <v>5</v>
+      </c>
+      <c r="D45" s="0">
+        <v>10</v>
+      </c>
+      <c r="E45" s="0">
+        <v>-88</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shampoo</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maharashtra</t>
+        </is>
+      </c>
+      <c r="C46" s="3">
+        <v>15</v>
+      </c>
+      <c r="D46" s="3">
+        <v>1</v>
+      </c>
+      <c r="E46" s="3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shampoo</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gujarat</t>
+        </is>
+      </c>
+      <c r="C47" s="3">
+        <v>11</v>
+      </c>
+      <c r="D47" s="3">
+        <v>3</v>
+      </c>
+      <c r="E47" s="3">
+        <v>-61</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shampoo</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="C48" s="3">
+        <v>10</v>
+      </c>
+      <c r="D48" s="3">
+        <v>2</v>
+      </c>
+      <c r="E48" s="3">
+        <v>-67</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shampoo</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delhi</t>
+        </is>
+      </c>
+      <c r="C49" s="3">
+        <v>7</v>
+      </c>
+      <c r="D49" s="3">
+        <v>2</v>
+      </c>
+      <c r="E49" s="3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shampoo</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Karnataka</t>
+        </is>
+      </c>
+      <c r="C50" s="3">
+        <v>6</v>
+      </c>
+      <c r="D50" s="3">
+        <v>3</v>
+      </c>
+      <c r="E50" s="3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shampoo</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Bengal</t>
+        </is>
+      </c>
+      <c r="C51" s="3">
+        <v>6</v>
+      </c>
+      <c r="D51" s="3">
+        <v>3</v>
+      </c>
+      <c r="E51" s="3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shampoo</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Haryana</t>
+        </is>
+      </c>
+      <c r="C52" s="3">
+        <v>6</v>
+      </c>
+      <c r="D52" s="3">
+        <v>2</v>
+      </c>
+      <c r="E52" s="3">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shampoo</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Punjab</t>
+        </is>
+      </c>
+      <c r="C53" s="3">
+        <v>6</v>
+      </c>
+      <c r="D53" s="3">
+        <v>1</v>
+      </c>
+      <c r="E53" s="3">
+        <v>-33</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Key insight: Uttar Pradesh and Maharashtra are the two largest under-penetrated states across BOTH categories -- the biggest white-space opportunity for distribution/visibility investment. Cross-check against the dashboard Distribution tab's store-level gap analysis for these states.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source: Nielsen National Urban MS Val readout, May'26 vintage, transcribed from the leadership deck on branch claude/retail-channel-performance-hz0q8h. This is total-market share vs named competitors, NOT the MT-vs-GT channel cut used in the other tabs of this workbook -- do not blend the two.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A55:H55"/>
+    <mergeCell ref="A57:H57"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
@@ -2975,7 +4188,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -3216,6 +4429,43 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Close UP/Maharashtra distribution white space</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Raise Nielsen share in UP &amp; Maharashtra toward category-contribution level</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RKAM / Zone Sales</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q3 FY27</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prioritize new-store/visibility spend in UP &amp; Maharashtra; both states are high category-contribution, low Nielsen-share in Facewash and Shampoo</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quarterly</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>